<commit_message>
chore: actualiza recorrido 2026-09-06T08:22Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/09/05 22:01:25</t>
+          <t>2026/09/05 23:01:38</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>165:59:47</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/09/05 22:31:21</t>
+          <t>2026/09/05 23:31:38</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>166:16:53</t>
+          <t>167:17:10</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/09/05 22:23:42</t>
+          <t>2026/09/05 23:23:13</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>166:00:02</t>
+          <t>166:59:33</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/09/05 22:42:06</t>
+          <t>2026/09/05 23:42:06</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>165:59:35</t>
+          <t>166:59:35</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/09/05 22:56:11</t>
+          <t>2026/09/05 23:56:11</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>165:59:35</t>
+          <t>166:59:35</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026/09/05 21:04:45</t>
+          <t>2026/09/05 23:04:45</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>164:00:00</t>
+          <t>166:00:00</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>2026/09/05 22:11:40</t>
+          <t>2026/09/05 23:11:21</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5413,7 +5413,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>125:27:26</t>
+          <t>126:27:07</t>
         </is>
       </c>
       <c r="L86" t="n">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026/09/05 22:46:44</t>
+          <t>2026/09/05 23:46:38</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>83:06:03</t>
+          <t>84:05:57</t>
         </is>
       </c>
       <c r="L133" t="n">
@@ -10472,7 +10472,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>2026/09/05 22:39:21</t>
+          <t>2026/09/05 23:39:21</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -10487,7 +10487,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>32:35:22</t>
+          <t>33:35:22</t>
         </is>
       </c>
       <c r="L172" t="n">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>2026/09/05 22:55:09</t>
+          <t>2026/09/05 23:55:35</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -10841,7 +10841,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>30:00:16</t>
+          <t>31:00:42</t>
         </is>
       </c>
       <c r="L178" t="n">
@@ -10944,26 +10944,26 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>2026/09/05 22:34:33</t>
+          <t>2026/09/05 23:04:45</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>-32.788598, -70.912005</t>
+          <t>-32.838394, -70.955539</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>-32.78860, -70.91200</t>
+          <t>-32.83839, -70.95554</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>24:30:46</t>
+          <t>25:00:58</t>
         </is>
       </c>
       <c r="L180" t="n">
-        <v>22.07</v>
+        <v>28.94</v>
       </c>
       <c r="M180" t="n">
         <v>0</v>
@@ -11216,7 +11216,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1062.24</v>
+        <v>1069.11</v>
       </c>
       <c r="C3" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-07T08:55Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N186"/>
+  <dimension ref="A1:N187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/09/06 22:01:38</t>
+          <t>2026/09/06 23:01:21</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>166:00:16</t>
+          <t>166:59:59</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/09/06 22:23:43</t>
+          <t>2026/09/06 23:22:46</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>166:01:05</t>
+          <t>167:00:08</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/09/06 22:40:43</t>
+          <t>2026/09/06 23:40:43</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>165:58:12</t>
+          <t>166:58:12</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/09/06 22:31:20</t>
+          <t>2026/09/06 23:31:38</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>165:47:12</t>
+          <t>166:47:30</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/09/06 22:56:06</t>
+          <t>2026/09/06 23:56:06</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>165:59:30</t>
+          <t>166:59:30</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/09/06 21:04:45</t>
+          <t>2026/09/06 23:04:45</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>164:00:00</t>
+          <t>166:00:00</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>2026/09/06 22:12:08</t>
+          <t>2026/09/06 23:12:11</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -5826,7 +5826,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>149:27:54</t>
+          <t>150:27:57</t>
         </is>
       </c>
       <c r="L93" t="n">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/09/06 22:46:25</t>
+          <t>2026/09/06 23:46:38</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>107:05:44</t>
+          <t>108:05:57</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>2026/09/06 22:39:31</t>
+          <t>2026/09/06 23:39:20</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -10723,7 +10723,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>56:35:32</t>
+          <t>57:35:21</t>
         </is>
       </c>
       <c r="L176" t="n">
@@ -11180,7 +11180,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>2026/09/06 21:38:57</t>
+          <t>2026/09/06 23:38:57</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -11195,7 +11195,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L184" t="n">
@@ -11323,6 +11323,65 @@
         <v>0</v>
       </c>
       <c r="N186" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCS-53</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>4</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>2026/09/06 21:06:07</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>-33.0873016, -71.3623533</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>-33.08730, -71.36235</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>2026/09/06 23:06:53</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>-33.0872433, -71.3622583</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>-33.08724, -71.36226</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>02:00:46</t>
+        </is>
+      </c>
+      <c r="L187" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M187" t="n">
+        <v>0</v>
+      </c>
+      <c r="N187" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11412,13 +11471,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>588.4299999999999</v>
+        <v>588.35</v>
       </c>
       <c r="C4" t="n">
         <v>78</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>140</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-08T08:36Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/09/07 22:40:43</t>
+          <t>2026/09/07 23:40:43</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>165:58:58</t>
+          <t>166:58:58</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -886,7 +886,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SLP20250627045-AC02</t>
+          <t>LPR20251V02900023-LL</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -894,7 +894,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -904,48 +904,48 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-34.205437, -70.677295</t>
+          <t>-33.899904, -71.429498</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-34.20544, -70.67730</t>
+          <t>-33.89990, -71.42950</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/09/02 08:55:46</t>
+          <t>2026/09/07 23:31:38</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>-34.205342, -70.680134</t>
+          <t>-33.89982, -71.429438</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>-34.20534, -70.68013</t>
+          <t>-33.89982, -71.42944</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>32:11:39</t>
+          <t>166:47:31</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>0.28</v>
+        <v>0.04</v>
       </c>
       <c r="M10" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LPR20251V02900023-LL</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -953,7 +953,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -963,42 +963,42 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-33.899904, -71.429498</t>
+          <t>-34.205437, -70.677295</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-33.89990, -71.42950</t>
+          <t>-34.20544, -70.67730</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/09/07 22:31:21</t>
+          <t>2026/09/02 08:55:46</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>-33.89982, -71.429438</t>
+          <t>-34.205342, -70.680134</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>-33.89982, -71.42944</t>
+          <t>-34.20534, -70.68013</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>165:47:14</t>
+          <t>32:11:39</t>
         </is>
       </c>
       <c r="L11" t="n">
-        <v>0.04</v>
+        <v>0.28</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/09/07 22:12:08</t>
+          <t>2026/09/07 23:11:45</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>165:24:39</t>
+          <t>166:24:16</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/09/07 22:56:06</t>
+          <t>2026/09/07 23:56:06</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>165:59:14</t>
+          <t>166:59:14</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>2026/09/07 22:39:21</t>
+          <t>2026/09/07 23:39:21</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>80:35:22</t>
+          <t>81:35:22</t>
         </is>
       </c>
       <c r="L150" t="n">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>2026/09/07 22:14:09</t>
+          <t>2026/09/07 23:14:08</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>07:01:17</t>
+          <t>08:01:16</t>
         </is>
       </c>
       <c r="L166" t="n">
@@ -10177,7 +10177,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>2026/09/07 21:21:38</t>
+          <t>2026/09/07 23:21:38</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>06:00:04</t>
+          <t>08:00:04</t>
         </is>
       </c>
       <c r="L167" t="n">
@@ -10236,7 +10236,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>2026/09/07 21:54:08</t>
+          <t>2026/09/07 23:54:08</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>04:01:06</t>
+          <t>06:01:06</t>
         </is>
       </c>
       <c r="L168" t="n">
@@ -10354,7 +10354,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>2026/09/07 21:15:37</t>
+          <t>2026/09/07 23:15:37</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -10369,7 +10369,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>02:01:00</t>
+          <t>04:01:00</t>
         </is>
       </c>
       <c r="L170" t="n">
@@ -10472,7 +10472,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>2026/09/07 21:48:03</t>
+          <t>2026/09/07 23:48:03</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -10487,7 +10487,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>01:49:03</t>
+          <t>03:49:03</t>
         </is>
       </c>
       <c r="L172" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-08T16:00Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -886,7 +886,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LPR20251V02900023-LL</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -894,7 +894,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -904,48 +904,48 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-33.899904, -71.429498</t>
+          <t>-34.205437, -70.677295</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-33.89990, -71.42950</t>
+          <t>-34.20544, -70.67730</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/09/07 23:31:38</t>
+          <t>2026/09/02 08:55:46</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>-33.89982, -71.429438</t>
+          <t>-34.205342, -70.680134</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>-33.89982, -71.42944</t>
+          <t>-34.20534, -70.68013</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>166:47:31</t>
+          <t>32:11:39</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>0.04</v>
+        <v>0.28</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SLP20250627045-AC02</t>
+          <t>LPR20251V02900023-LL</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -953,7 +953,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -963,42 +963,42 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-34.205437, -70.677295</t>
+          <t>-33.899904, -71.429498</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-34.20544, -70.67730</t>
+          <t>-33.89990, -71.42950</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/09/02 08:55:46</t>
+          <t>2026/09/07 23:31:38</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>-34.205342, -70.680134</t>
+          <t>-33.89982, -71.429438</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>-34.20534, -70.68013</t>
+          <t>-33.89982, -71.42944</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>32:11:39</t>
+          <t>166:47:31</t>
         </is>
       </c>
       <c r="L11" t="n">
-        <v>0.28</v>
+        <v>0.04</v>
       </c>
       <c r="M11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-09T08:38Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/09/08 22:40:35</t>
+          <t>2026/09/08 23:40:35</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>165:58:50</t>
+          <t>166:58:50</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/09/08 22:31:38</t>
+          <t>2026/09/08 23:31:21</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>165:47:38</t>
+          <t>166:47:21</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/09/08 22:08:45</t>
+          <t>2026/09/08 23:09:09</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>165:24:13</t>
+          <t>166:24:37</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/09/08 22:56:11</t>
+          <t>2026/09/08 23:56:11</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>165:59:19</t>
+          <t>166:59:19</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -8938,7 +8938,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>2026/09/08 22:13:38</t>
+          <t>2026/09/08 23:13:18</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>104:09:39</t>
+          <t>105:09:19</t>
         </is>
       </c>
       <c r="L146" t="n">
@@ -9351,7 +9351,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>2026/09/08 22:46:52</t>
+          <t>2026/09/08 23:46:52</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>43:00:24</t>
+          <t>44:00:24</t>
         </is>
       </c>
       <c r="L153" t="n">
@@ -10354,7 +10354,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>2026/09/08 22:35:23</t>
+          <t>2026/09/08 23:35:23</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -10369,7 +10369,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>09:45:07</t>
+          <t>10:45:07</t>
         </is>
       </c>
       <c r="L170" t="n">
@@ -10590,7 +10590,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>2026/09/08 22:57:30</t>
+          <t>2026/09/08 23:57:30</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -10605,7 +10605,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>09:01:08</t>
+          <t>10:01:08</t>
         </is>
       </c>
       <c r="L174" t="n">
@@ -10649,7 +10649,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>2026/09/08 22:28:01</t>
+          <t>2026/09/08 23:28:01</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>07:01:16</t>
+          <t>08:01:16</t>
         </is>
       </c>
       <c r="L175" t="n">
@@ -10885,7 +10885,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>2026/09/08 21:09:50</t>
+          <t>2026/09/08 23:09:50</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -10900,7 +10900,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>02:00:58</t>
+          <t>04:00:58</t>
         </is>
       </c>
       <c r="L179" t="n">
@@ -11003,7 +11003,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>2026/09/08 21:31:52</t>
+          <t>2026/09/08 23:31:52</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>02:00:02</t>
+          <t>04:00:02</t>
         </is>
       </c>
       <c r="L181" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-10T08:39Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N155"/>
+  <dimension ref="A1:N156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/09/09 22:31:21</t>
+          <t>2026/09/09 23:31:25</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>166:00:00</t>
+          <t>167:00:04</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/09/09 22:40:35</t>
+          <t>2026/09/09 23:40:35</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>165:58:54</t>
+          <t>166:58:54</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/09/09 22:56:11</t>
+          <t>2026/09/09 23:56:11</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>166:00:02</t>
+          <t>167:00:02</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>2026/09/09 22:35:22</t>
+          <t>2026/09/09 23:35:03</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>33:45:06</t>
+          <t>34:44:47</t>
         </is>
       </c>
       <c r="L142" t="n">
@@ -8938,7 +8938,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>2026/09/09 22:54:33</t>
+          <t>2026/09/09 23:54:22</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>32:58:11</t>
+          <t>33:58:00</t>
         </is>
       </c>
       <c r="L146" t="n">
@@ -8997,7 +8997,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>2026/09/09 22:25:00</t>
+          <t>2026/09/09 23:24:47</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>30:58:15</t>
+          <t>31:58:02</t>
         </is>
       </c>
       <c r="L147" t="n">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2026/09/09 21:34:28</t>
+          <t>2026/09/09 23:34:28</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L154" t="n">
@@ -9494,6 +9494,65 @@
         <v>0</v>
       </c>
       <c r="N155" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>5</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>2026/09/09 21:27:13</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>-33.4366466, -70.6296616</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>-33.43665, -70.62966</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>2026/09/09 23:29:06</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>-33.4366466, -70.6296616</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>-33.43665, -70.62966</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>02:01:53</t>
+        </is>
+      </c>
+      <c r="L156" t="n">
+        <v>0</v>
+      </c>
+      <c r="M156" t="n">
+        <v>0</v>
+      </c>
+      <c r="N156" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9792,13 +9851,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>392.32</v>
+        <v>392.28</v>
       </c>
       <c r="C15" t="n">
         <v>31</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>138</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-11T08:34Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/09/10 22:06:21</t>
+          <t>2026/09/10 23:06:36</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>165:54:42</t>
+          <t>166:54:57</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/09/10 22:31:52</t>
+          <t>2026/09/10 23:31:30</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>166:00:31</t>
+          <t>167:00:09</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/09/10 22:41:02</t>
+          <t>2026/09/10 23:41:02</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>165:59:21</t>
+          <t>166:59:21</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/09/10 22:56:10</t>
+          <t>2026/09/10 23:56:10</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>166:00:01</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -7699,7 +7699,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>2026/09/10 22:34:38</t>
+          <t>2026/09/10 23:34:47</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>57:44:22</t>
+          <t>58:44:31</t>
         </is>
       </c>
       <c r="L125" t="n">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/09/10 22:54:30</t>
+          <t>2026/09/10 23:54:17</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>56:58:08</t>
+          <t>57:57:55</t>
         </is>
       </c>
       <c r="L130" t="n">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026/09/10 22:09:33</t>
+          <t>2026/09/10 23:09:54</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>30:44:56</t>
+          <t>31:45:17</t>
         </is>
       </c>
       <c r="L136" t="n">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2026/09/10 21:42:06</t>
+          <t>2026/09/10 23:42:06</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>10:00:44</t>
+          <t>12:00:44</t>
         </is>
       </c>
       <c r="L137" t="n">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>2026/09/10 21:37:12</t>
+          <t>2026/09/10 23:37:12</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>04:00:17</t>
+          <t>06:00:17</t>
         </is>
       </c>
       <c r="L138" t="n">
@@ -8525,7 +8525,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>2026/09/10 21:47:06</t>
+          <t>2026/09/10 23:47:06</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -8540,7 +8540,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L139" t="n">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/09/10 21:40:33</t>
+          <t>2026/09/10 23:40:33</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>02:00:20</t>
+          <t>04:00:20</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>2026/09/10 21:43:06</t>
+          <t>2026/09/10 23:43:06</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>02:00:35</t>
+          <t>04:00:35</t>
         </is>
       </c>
       <c r="L141" t="n">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>2026/09/10 21:54:59</t>
+          <t>2026/09/10 23:54:59</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>02:01:24</t>
+          <t>04:01:24</t>
         </is>
       </c>
       <c r="L142" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-12T08:22Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/09/11 22:31:27</t>
+          <t>2026/09/11 23:31:54</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>165:59:50</t>
+          <t>167:00:17</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/09/11 22:41:02</t>
+          <t>2026/09/11 23:41:02</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>165:58:56</t>
+          <t>166:58:56</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/09/11 22:56:10</t>
+          <t>2026/09/11 23:56:10</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>165:59:59</t>
+          <t>166:59:59</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -5575,7 +5575,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>2026/09/11 22:34:21</t>
+          <t>2026/09/11 23:34:40</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>81:44:05</t>
+          <t>82:44:24</t>
         </is>
       </c>
       <c r="L89" t="n">
@@ -5988,7 +5988,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>2026/09/11 22:57:48</t>
+          <t>2026/09/11 23:57:51</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6003,7 +6003,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>79:31:03</t>
+          <t>80:31:06</t>
         </is>
       </c>
       <c r="L96" t="n">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026/09/11 21:14:47</t>
+          <t>2026/09/11 23:14:47</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>02:01:00</t>
+          <t>04:01:00</t>
         </is>
       </c>
       <c r="L123" t="n">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/09/11 21:43:56</t>
+          <t>2026/09/11 23:43:56</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L124" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-13T08:56Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N127"/>
+  <dimension ref="A1:N128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/09/12 22:31:38</t>
+          <t>2026/09/12 23:31:38</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>166:00:00</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/09/12 22:41:10</t>
+          <t>2026/09/12 23:41:10</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>165:59:04</t>
+          <t>166:59:04</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/09/12 22:56:08</t>
+          <t>2026/09/12 23:56:08</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>165:59:57</t>
+          <t>166:59:57</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>2026/09/12 22:57:15</t>
+          <t>2026/09/12 23:57:38</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>103:30:30</t>
+          <t>104:30:53</t>
         </is>
       </c>
       <c r="L99" t="n">
@@ -7842,6 +7842,65 @@
         <v>0</v>
       </c>
       <c r="N127" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TGPS-77</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>7</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>2026/09/12 21:39:50</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>-32.7976249, -70.8871033</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>-32.79762, -70.88710</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>2026/09/12 23:40:06</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>-32.7976249, -70.8871033</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>-32.79762, -70.88710</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>02:00:16</t>
+        </is>
+      </c>
+      <c r="L128" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" t="n">
+        <v>0</v>
+      </c>
+      <c r="N128" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7893,13 +7952,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1894.52</v>
+        <v>1894.49</v>
       </c>
       <c r="C2" t="n">
         <v>71</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>144</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-14T09:34Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/09/13 22:31:26</t>
+          <t>2026/09/13 23:31:38</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>165:59:48</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/09/13 22:41:10</t>
+          <t>2026/09/13 23:41:10</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>166:00:27</t>
+          <t>167:00:27</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/09/13 22:56:08</t>
+          <t>2026/09/13 23:56:08</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>166:00:02</t>
+          <t>167:00:02</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>2026/09/13 22:57:15</t>
+          <t>2026/09/13 23:57:38</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6121,7 +6121,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>127:30:30</t>
+          <t>128:30:53</t>
         </is>
       </c>
       <c r="L98" t="n">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>2026/09/13 22:34:39</t>
+          <t>2026/09/13 23:34:24</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>43:59:03</t>
+          <t>44:58:48</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/09/13 21:28:57</t>
+          <t>2026/09/13 23:28:57</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="L124" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-14T22:56Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -2243,7 +2243,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>LPR20251H02800016-STL</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2261,48 +2261,48 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>-33.0873333, -71.3622983</t>
+          <t>-34.042559, -70.681776</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>-33.08733, -71.36230</t>
+          <t>-34.04256, -70.68178</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2026/09/07 11:20:40</t>
+          <t>2026/09/07 14:24:10</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>-33.45388, -71.30113</t>
+          <t>-34.042735, -70.681661</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>-33.45388, -71.30113</t>
+          <t>-34.04274, -70.68166</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>01:53:52</t>
+          <t>04:57:22</t>
         </is>
       </c>
       <c r="L33" t="n">
-        <v>62.66</v>
+        <v>0.03</v>
       </c>
       <c r="M33" t="n">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>LPR20251H02800016-STL</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2320,42 +2320,42 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>-34.042559, -70.681776</t>
+          <t>-33.0873333, -71.3622983</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>-34.04256, -70.68178</t>
+          <t>-33.08733, -71.36230</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026/09/07 14:24:10</t>
+          <t>2026/09/07 11:20:40</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>-34.042735, -70.681661</t>
+          <t>-33.45388, -71.30113</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>-34.04274, -70.68166</t>
+          <t>-33.45388, -71.30113</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>04:57:22</t>
+          <t>01:53:52</t>
         </is>
       </c>
       <c r="L34" t="n">
-        <v>0.03</v>
+        <v>62.66</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="N34" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-15T09:11Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/09/14 22:31:38</t>
+          <t>2026/09/14 23:31:38</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>166:00:00</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/09/14 22:41:51</t>
+          <t>2026/09/14 23:41:51</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>166:01:08</t>
+          <t>167:01:08</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/09/14 22:56:13</t>
+          <t>2026/09/14 23:56:13</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>166:00:07</t>
+          <t>167:00:07</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -4454,7 +4454,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>2026/09/14 22:57:17</t>
+          <t>2026/09/14 23:57:39</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4469,7 +4469,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>151:30:32</t>
+          <t>152:30:54</t>
         </is>
       </c>
       <c r="L70" t="n">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2026/09/14 22:34:21</t>
+          <t>2026/09/14 23:34:38</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -7301,7 +7301,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>67:58:45</t>
+          <t>68:59:02</t>
         </is>
       </c>
       <c r="L118" t="n">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/09/14 22:45:08</t>
+          <t>2026/09/14 23:45:08</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>06:01:46</t>
+          <t>07:01:46</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>2026/09/14 21:51:38</t>
+          <t>2026/09/14 23:51:38</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L141" t="n">
@@ -8938,7 +8938,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>2026/09/14 21:41:40</t>
+          <t>2026/09/14 23:41:40</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>02:00:52</t>
+          <t>04:00:52</t>
         </is>
       </c>
       <c r="L146" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-16T09:04Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/09/15 22:57:39</t>
+          <t>2026/09/15 23:57:15</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>166:29:38</t>
+          <t>167:29:14</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -9292,7 +9292,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>2026/09/15 21:47:19</t>
+          <t>2026/09/15 23:47:19</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L152" t="n">
@@ -9351,7 +9351,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>2026/09/15 21:53:13</t>
+          <t>2026/09/15 23:53:13</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>04:01:06</t>
+          <t>06:01:06</t>
         </is>
       </c>
       <c r="L153" t="n">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2026/09/15 21:55:56</t>
+          <t>2026/09/15 23:55:56</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L154" t="n">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>2026/09/15 21:59:55</t>
+          <t>2026/09/15 23:59:55</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>02:00:08</t>
+          <t>04:00:08</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -9859,7 +9859,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>586.8099999999999</v>
+        <v>593.63</v>
       </c>
       <c r="C3" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-17T09:13Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N165"/>
+  <dimension ref="A1:N166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/09/16 22:46:35</t>
+          <t>2026/09/16 23:46:08</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>30:39:43</t>
+          <t>31:39:16</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -9469,7 +9469,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>2026/09/16 21:54:00</t>
+          <t>2026/09/16 23:54:00</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>06:00:03</t>
+          <t>08:00:03</t>
         </is>
       </c>
       <c r="L155" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/09/16 21:37:48</t>
+          <t>2026/09/16 23:37:48</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>04:00:04</t>
+          <t>06:00:04</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>2026/09/16 21:45:51</t>
+          <t>2026/09/16 23:45:51</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>02:00:52</t>
+          <t>04:00:52</t>
         </is>
       </c>
       <c r="L163" t="n">
@@ -10059,32 +10059,91 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>2026/09/16 23:21:06</t>
+          <t>2026/09/16 23:19:53</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>-33.5079416, -70.6288266</t>
+          <t>-33.5078883, -70.6289333</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>-33.50794, -70.62883</t>
+          <t>-33.50789, -70.62893</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>00:53:49</t>
+          <t>00:52:36</t>
         </is>
       </c>
       <c r="L165" t="n">
-        <v>12.14</v>
+        <v>12.13</v>
       </c>
       <c r="M165" t="n">
         <v>83</v>
       </c>
       <c r="N165" t="n">
         <v>29</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>OPEL COMBO</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>9</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>2026/09/16 23:21:06</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>-33.5079416, -70.6288266</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>-33.50794, -70.62883</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>2026/09/16 23:43:06</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>-33.51385, -70.6382499</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>-33.51385, -70.63825</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>00:22:00</t>
+        </is>
+      </c>
+      <c r="L166" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="M166" t="n">
+        <v>18</v>
+      </c>
+      <c r="N166" t="n">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -10401,10 +10460,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>184.09</v>
+        <v>185.68</v>
       </c>
       <c r="C16" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-18T08:45Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -7640,7 +7640,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/09/17 22:23:58</t>
+          <t>2026/09/17 23:24:20</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>55:07:04</t>
+          <t>56:07:26</t>
         </is>
       </c>
       <c r="L124" t="n">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/09/17 22:46:23</t>
+          <t>2026/09/17 23:46:38</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>54:39:31</t>
+          <t>55:39:46</t>
         </is>
       </c>
       <c r="L130" t="n">
@@ -9469,7 +9469,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>2026/09/17 21:33:04</t>
+          <t>2026/09/17 23:33:04</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>03:35:56</t>
+          <t>05:35:56</t>
         </is>
       </c>
       <c r="L155" t="n">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>2026/09/17 21:31:13</t>
+          <t>2026/09/17 23:31:13</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>02:01:00</t>
+          <t>04:01:00</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -9918,7 +9918,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>635.0599999999999</v>
+        <v>636.86</v>
       </c>
       <c r="C3" t="n">
         <v>15</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-19T08:32Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N163"/>
+  <dimension ref="A1:N161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/09/18 22:42:12</t>
+          <t>2026/09/18 23:42:12</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>166:01:10</t>
+          <t>167:01:10</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/09/18 22:56:13</t>
+          <t>2026/09/18 23:56:13</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>166:00:03</t>
+          <t>167:00:03</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>2026/09/18 22:22:57</t>
+          <t>2026/09/18 23:22:59</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>83:22:34</t>
+          <t>84:22:36</t>
         </is>
       </c>
       <c r="L108" t="n">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>2026/09/18 22:23:57</t>
+          <t>2026/09/18 23:24:20</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>79:07:03</t>
+          <t>80:07:26</t>
         </is>
       </c>
       <c r="L121" t="n">
@@ -9351,7 +9351,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>2026/09/18 21:16:39</t>
+          <t>2026/09/18 23:16:39</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>26:52:42</t>
+          <t>28:52:42</t>
         </is>
       </c>
       <c r="L153" t="n">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>2026/09/18 22:46:31</t>
+          <t>2026/09/18 23:46:15</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>19:00:13</t>
+          <t>19:59:57</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026/09/18 21:25:59</t>
+          <t>2026/09/18 23:25:59</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="L159" t="n">
@@ -9736,11 +9736,11 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>SUZUKI CARRY SKDB-52</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
@@ -9749,37 +9749,37 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>2026/09/18 17:57:23</t>
+          <t>2026/09/18 19:47:53</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>-33.4584983, -70.6632966</t>
+          <t>-32.7976083, -70.8870616</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>-33.45850, -70.66330</t>
+          <t>-32.79761, -70.88706</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/09/18 21:57:25</t>
+          <t>2026/09/18 23:48:02</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>-33.4584983, -70.6632966</t>
+          <t>-32.7976083, -70.8870616</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>-33.45850, -70.66330</t>
+          <t>-32.79761, -70.88706</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>04:00:02</t>
+          <t>04:00:09</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -9795,11 +9795,11 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TGPS-77</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
@@ -9808,37 +9808,37 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>2026/09/18 19:47:53</t>
+          <t>2026/09/18 19:53:11</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>-32.7976083, -70.8870616</t>
+          <t>-33.0871666, -71.3621533</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>-32.79761, -70.88706</t>
+          <t>-33.08717, -71.36215</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>2026/09/18 21:48:02</t>
+          <t>2026/09/18 23:53:11</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>-32.7976083, -70.8870616</t>
+          <t>-33.0871666, -71.3621533</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>-32.79761, -70.88706</t>
+          <t>-33.08717, -71.36215</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>02:00:09</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L161" t="n">
@@ -9848,124 +9848,6 @@
         <v>0</v>
       </c>
       <c r="N161" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
-        </is>
-      </c>
-      <c r="C162" t="n">
-        <v>3</v>
-      </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>Paradas</t>
-        </is>
-      </c>
-      <c r="E162" t="inlineStr">
-        <is>
-          <t>2026/09/18 19:53:11</t>
-        </is>
-      </c>
-      <c r="F162" t="inlineStr">
-        <is>
-          <t>-33.0871666, -71.3621533</t>
-        </is>
-      </c>
-      <c r="G162" t="inlineStr">
-        <is>
-          <t>-33.08717, -71.36215</t>
-        </is>
-      </c>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>2026/09/18 21:53:11</t>
-        </is>
-      </c>
-      <c r="I162" t="inlineStr">
-        <is>
-          <t>-33.0871666, -71.3621533</t>
-        </is>
-      </c>
-      <c r="J162" t="inlineStr">
-        <is>
-          <t>-33.08717, -71.36215</t>
-        </is>
-      </c>
-      <c r="K162" t="inlineStr">
-        <is>
-          <t>02:00:00</t>
-        </is>
-      </c>
-      <c r="L162" t="n">
-        <v>0</v>
-      </c>
-      <c r="M162" t="n">
-        <v>0</v>
-      </c>
-      <c r="N162" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>CHANGAN HUNTER TKCL-70</t>
-        </is>
-      </c>
-      <c r="C163" t="n">
-        <v>2</v>
-      </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>Paradas</t>
-        </is>
-      </c>
-      <c r="E163" t="inlineStr">
-        <is>
-          <t>2026/09/18 21:22:13</t>
-        </is>
-      </c>
-      <c r="F163" t="inlineStr">
-        <is>
-          <t>-32.841563, -70.936737</t>
-        </is>
-      </c>
-      <c r="G163" t="inlineStr">
-        <is>
-          <t>-32.84156, -70.93674</t>
-        </is>
-      </c>
-      <c r="H163" t="inlineStr">
-        <is>
-          <t>2026/09/18 22:16:03</t>
-        </is>
-      </c>
-      <c r="I163" t="inlineStr">
-        <is>
-          <t>-32.841698, -70.936857</t>
-        </is>
-      </c>
-      <c r="J163" t="inlineStr">
-        <is>
-          <t>-32.84170, -70.93686</t>
-        </is>
-      </c>
-      <c r="K163" t="inlineStr">
-        <is>
-          <t>00:53:50</t>
-        </is>
-      </c>
-      <c r="L163" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="M163" t="n">
-        <v>0</v>
-      </c>
-      <c r="N163" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10036,13 +9918,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>477</v>
+        <v>478.82</v>
       </c>
       <c r="C3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>18</v>
@@ -10340,13 +10222,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>935.5700000000001</v>
+        <v>1000.2</v>
       </c>
       <c r="C19" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>136</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-20T09:04Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/09/19 22:42:12</t>
+          <t>2026/09/19 23:42:12</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>166:01:02</t>
+          <t>167:01:02</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/09/19 22:56:13</t>
+          <t>2026/09/19 23:56:13</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>166:00:05</t>
+          <t>167:00:05</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>2026/09/19 21:58:11</t>
+          <t>2026/09/19 23:58:11</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -9897,7 +9897,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="L162" t="n">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>2026/09/19 21:33:18</t>
+          <t>2026/09/19 23:33:18</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L164" t="n">
@@ -10272,7 +10272,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>470.64</v>
+        <v>472.52</v>
       </c>
       <c r="C3" t="n">
         <v>18</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-21T09:36Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/09/20 22:40:44</t>
+          <t>2026/09/20 23:40:44</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>165:59:34</t>
+          <t>166:59:34</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/09/20 22:56:09</t>
+          <t>2026/09/20 23:56:09</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>166:00:01</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>2026/09/20 22:22:38</t>
+          <t>2026/09/20 23:23:15</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7124,7 +7124,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>131:22:15</t>
+          <t>132:22:52</t>
         </is>
       </c>
       <c r="L115" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/09/20 21:33:18</t>
+          <t>2026/09/20 23:33:18</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>26:00:00</t>
+          <t>28:00:00</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -10059,7 +10059,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>2026/09/20 21:30:21</t>
+          <t>2026/09/20 23:30:21</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -10074,7 +10074,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>02:00:37</t>
+          <t>04:00:37</t>
         </is>
       </c>
       <c r="L165" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-22T09:01Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/09/21 22:40:44</t>
+          <t>2026/09/21 23:40:44</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>165:58:53</t>
+          <t>166:58:53</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/09/21 22:56:09</t>
+          <t>2026/09/21 23:56:09</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>165:59:56</t>
+          <t>166:59:56</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -3392,7 +3392,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>2026/09/21 22:23:31</t>
+          <t>2026/09/21 23:22:38</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>155:23:08</t>
+          <t>156:22:15</t>
         </is>
       </c>
       <c r="L52" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026/09/21 22:32:56</t>
+          <t>2026/09/21 23:32:29</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>31:00:24</t>
+          <t>31:59:57</t>
         </is>
       </c>
       <c r="L159" t="n">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>2026/09/21 21:49:51</t>
+          <t>2026/09/21 23:49:51</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -9838,7 +9838,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>12:00:28</t>
+          <t>14:00:28</t>
         </is>
       </c>
       <c r="L161" t="n">
@@ -10472,7 +10472,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>2026/09/21 21:23:01</t>
+          <t>2026/09/21 23:23:01</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -10487,7 +10487,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L172" t="n">
@@ -10531,7 +10531,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>2026/09/21 21:39:42</t>
+          <t>2026/09/21 23:39:42</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -10546,7 +10546,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L173" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-23T09:05Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/09/22 22:56:11</t>
+          <t>2026/09/22 23:56:11</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>166:50:43</t>
+          <t>167:50:43</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -7404,7 +7404,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026/09/22 21:49:51</t>
+          <t>2026/09/22 23:49:51</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>36:00:28</t>
+          <t>38:00:28</t>
         </is>
       </c>
       <c r="L120" t="n">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026/09/22 22:22:51</t>
+          <t>2026/09/22 23:23:07</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>20:00:24</t>
+          <t>21:00:40</t>
         </is>
       </c>
       <c r="L133" t="n">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>2026/09/22 21:39:43</t>
+          <t>2026/09/22 23:39:43</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>05:25:27</t>
+          <t>07:25:27</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026/09/22 22:32:25</t>
+          <t>2026/09/22 23:32:25</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>06:01:37</t>
+          <t>07:01:37</t>
         </is>
       </c>
       <c r="L159" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/09/22 21:36:09</t>
+          <t>2026/09/22 23:36:09</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>2026/09/22 21:57:54</t>
+          <t>2026/09/22 23:57:54</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -9897,7 +9897,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>02:01:09</t>
+          <t>04:01:09</t>
         </is>
       </c>
       <c r="L162" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-24T08:59Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -737,7 +737,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/09/23 22:56:11</t>
+          <t>2026/09/23 23:56:11</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>166:48:13</t>
+          <t>167:48:13</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -6755,7 +6755,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>2026/09/23 22:22:55</t>
+          <t>2026/09/23 23:22:52</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -6770,7 +6770,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>44:00:28</t>
+          <t>45:00:25</t>
         </is>
       </c>
       <c r="L109" t="n">
@@ -7876,7 +7876,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>2026/09/23 22:57:17</t>
+          <t>2026/09/23 23:57:09</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>32:56:22</t>
+          <t>33:56:14</t>
         </is>
       </c>
       <c r="L128" t="n">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026/09/23 22:51:55</t>
+          <t>2026/09/23 23:51:55</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -8776,7 +8776,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>11:01:00</t>
+          <t>12:01:00</t>
         </is>
       </c>
       <c r="L143" t="n">
@@ -8997,7 +8997,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>2026/09/23 22:58:36</t>
+          <t>2026/09/23 23:58:37</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>08:01:13</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="L147" t="n">
@@ -9115,7 +9115,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>2026/09/23 21:15:34</t>
+          <t>2026/09/23 23:15:34</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9130,7 +9130,7 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>06:00:20</t>
+          <t>08:00:20</t>
         </is>
       </c>
       <c r="L149" t="n">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2026/09/23 21:14:09</t>
+          <t>2026/09/23 23:14:09</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L154" t="n">
@@ -9469,7 +9469,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>2026/09/23 21:22:13</t>
+          <t>2026/09/23 23:22:13</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>02:00:22</t>
+          <t>04:00:22</t>
         </is>
       </c>
       <c r="L155" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-25T09:23Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -619,7 +619,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/09/24 22:57:32</t>
+          <t>2026/09/24 23:57:32</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>166:49:34</t>
+          <t>167:49:34</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -6991,7 +6991,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>2026/09/24 22:57:38</t>
+          <t>2026/09/24 23:57:15</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7006,7 +7006,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>56:56:43</t>
+          <t>57:56:20</t>
         </is>
       </c>
       <c r="L113" t="n">
@@ -8997,7 +8997,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>2026/09/24 22:42:20</t>
+          <t>2026/09/24 23:42:20</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>08:24:42</t>
+          <t>09:24:42</t>
         </is>
       </c>
       <c r="L147" t="n">
@@ -9292,7 +9292,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>2026/09/24 21:31:32</t>
+          <t>2026/09/24 23:31:32</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L152" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-26T09:07Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/09/25 22:57:32</t>
+          <t>2026/09/25 23:57:32</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>166:01:19</t>
+          <t>167:01:19</t>
         </is>
       </c>
       <c r="L14" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-27T09:49Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/09/26 22:56:06</t>
+          <t>2026/09/26 23:56:06</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>165:59:53</t>
+          <t>166:59:53</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2026/09/26 22:50:57</t>
+          <t>2026/09/26 23:50:31</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>151:18:25</t>
+          <t>152:17:59</t>
         </is>
       </c>
       <c r="L38" t="n">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>2026/09/26 22:46:17</t>
+          <t>2026/09/26 23:46:41</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>35:48:45</t>
+          <t>36:49:09</t>
         </is>
       </c>
       <c r="L164" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-28T10:34Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/09/27 22:50:57</t>
+          <t>2026/09/27 23:50:29</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>166:18:24</t>
+          <t>167:17:56</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/09/27 22:56:06</t>
+          <t>2026/09/27 23:56:06</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>165:59:57</t>
+          <t>166:59:57</t>
         </is>
       </c>
       <c r="L14" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-29T10:24Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N162"/>
+  <dimension ref="A1:N165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/09/28 19:51:36</t>
+          <t>2026/09/28 23:51:14</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>163:19:03</t>
+          <t>167:18:41</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/09/28 19:56:10</t>
+          <t>2026/09/28 23:56:10</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>163:00:01</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026/09/28 19:22:30</t>
+          <t>2026/09/28 23:22:33</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>161:00:03</t>
+          <t>165:00:06</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>2026/09/28 19:43:31</t>
+          <t>2026/09/28 23:43:31</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>153:00:56</t>
+          <t>157:00:56</t>
         </is>
       </c>
       <c r="L53" t="n">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026/09/28 19:15:34</t>
+          <t>2026/09/28 23:15:34</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -8776,7 +8776,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>124:00:20</t>
+          <t>128:00:20</t>
         </is>
       </c>
       <c r="L143" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026/09/28 19:46:21</t>
+          <t>2026/09/28 23:46:48</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>16:00:06</t>
+          <t>20:00:33</t>
         </is>
       </c>
       <c r="L159" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/09/28 18:33:38</t>
+          <t>2026/09/28 22:33:38</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>2026/09/28 18:34:03</t>
+          <t>2026/09/28 22:34:03</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -9838,7 +9838,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L161" t="n">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>2026/09/28 19:21:37</t>
+          <t>2026/09/28 23:21:37</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -9897,7 +9897,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>00:49:41</t>
+          <t>04:49:41</t>
         </is>
       </c>
       <c r="L162" t="n">
@@ -9907,6 +9907,183 @@
         <v>0</v>
       </c>
       <c r="N162" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TGPS-77</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>9</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>2026/09/28 19:08:50</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>-32.7975783, -70.8870583</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>-32.79758, -70.88706</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>2026/09/28 22:31:01</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>-32.7975783, -70.8870583</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>-32.79758, -70.88706</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>03:22:11</t>
+        </is>
+      </c>
+      <c r="L163" t="n">
+        <v>0</v>
+      </c>
+      <c r="M163" t="n">
+        <v>0</v>
+      </c>
+      <c r="N163" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>14</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>2026/09/28 20:29:38</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>-33.4761233, -70.6985033</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>-33.47612, -70.69850</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>2026/09/28 22:29:38</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>-33.4761233, -70.6985033</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>-33.47612, -70.69850</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L164" t="n">
+        <v>0</v>
+      </c>
+      <c r="M164" t="n">
+        <v>0</v>
+      </c>
+      <c r="N164" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>SUZUKI CARRY SKDB-52</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>12</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>2026/09/28 20:41:53</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>-32.8791716, -70.6088033</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>-32.87917, -70.60880</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>2026/09/28 22:41:53</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>-32.8791716, -70.6088033</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>-32.87917, -70.60880</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L165" t="n">
+        <v>0</v>
+      </c>
+      <c r="M165" t="n">
+        <v>0</v>
+      </c>
+      <c r="N165" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9958,13 +10135,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1611.09</v>
+        <v>1611.06</v>
       </c>
       <c r="C2" t="n">
         <v>57</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>146</v>
@@ -10186,13 +10363,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1304.26</v>
+        <v>1322.27</v>
       </c>
       <c r="C14" t="n">
         <v>70</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>128</v>
@@ -10281,13 +10458,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>725.65</v>
+        <v>736.84</v>
       </c>
       <c r="C19" t="n">
         <v>75</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" t="n">
         <v>134</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-06T11:01Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N145"/>
+  <dimension ref="A1:N147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026/10/05 20:31:37</t>
+          <t>2026/10/05 23:31:38</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>162:00:17</t>
+          <t>165:00:18</t>
         </is>
       </c>
       <c r="L22" t="n">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>2026/10/05 20:46:26</t>
+          <t>2026/10/05 23:46:20</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7124,7 +7124,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>100:39:32</t>
+          <t>103:39:26</t>
         </is>
       </c>
       <c r="L115" t="n">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026/10/05 20:56:50</t>
+          <t>2026/10/05 23:56:50</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>81:51:10</t>
+          <t>84:51:10</t>
         </is>
       </c>
       <c r="L123" t="n">
@@ -7876,7 +7876,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>2026/10/05 20:18:49</t>
+          <t>2026/10/05 22:18:49</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>76:00:00</t>
+          <t>78:00:00</t>
         </is>
       </c>
       <c r="L128" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/10/05 20:11:39</t>
+          <t>2026/10/05 23:11:55</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>66:00:00</t>
+          <t>69:00:16</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026/10/05 20:09:17</t>
+          <t>2026/10/05 23:09:15</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>11:59:56</t>
+          <t>14:59:54</t>
         </is>
       </c>
       <c r="L134" t="n">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>2026/10/05 20:24:31</t>
+          <t>2026/10/05 23:24:31</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>03:01:14</t>
+          <t>06:01:14</t>
         </is>
       </c>
       <c r="L141" t="n">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>2026/10/05 20:30:20</t>
+          <t>2026/10/05 22:30:20</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>02:20:46</t>
+          <t>04:20:46</t>
         </is>
       </c>
       <c r="L142" t="n">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026/10/05 20:23:51</t>
+          <t>2026/10/05 22:23:51</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -8776,7 +8776,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>02:00:06</t>
+          <t>04:00:06</t>
         </is>
       </c>
       <c r="L143" t="n">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>2026/10/05 20:27:19</t>
+          <t>2026/10/05 22:27:19</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -8835,7 +8835,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L144" t="n">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>2026/10/05 20:29:04</t>
+          <t>2026/10/05 22:29:04</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L145" t="n">
@@ -8904,6 +8904,124 @@
         <v>0</v>
       </c>
       <c r="N145" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>JAC X200 SJTJ-50</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>12</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>2026/10/05 19:07:16</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>-32.7431783, -70.7296866</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>-32.74318, -70.72969</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>2026/10/05 23:08:49</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>-32.7430966, -70.7297466</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>-32.74310, -70.72975</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>04:01:33</t>
+        </is>
+      </c>
+      <c r="L146" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M146" t="n">
+        <v>0</v>
+      </c>
+      <c r="N146" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>3</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>2026/10/05 20:36:04</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>-33.4363166, -70.6293333</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>-33.43632, -70.62933</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>2026/10/05 22:36:55</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>-33.4364216, -70.62921</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>-33.43642, -70.62921</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>02:00:51</t>
+        </is>
+      </c>
+      <c r="L147" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M147" t="n">
+        <v>0</v>
+      </c>
+      <c r="N147" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9012,13 +9130,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>762.33</v>
+        <v>762.22</v>
       </c>
       <c r="C5" t="n">
         <v>46</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>131</v>
@@ -9202,13 +9320,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>658.6799999999999</v>
+        <v>658.6</v>
       </c>
       <c r="C15" t="n">
         <v>29</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>139</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-13T11:25Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N133"/>
+  <dimension ref="A1:N134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/10/12 20:56:21</t>
+          <t>2026/10/12 23:56:38</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>164:47:07</t>
+          <t>167:47:24</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/10/12 20:57:28</t>
+          <t>2026/10/12 23:57:28</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>164:00:38</t>
+          <t>167:00:38</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -5752,7 +5752,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>2026/10/12 21:01:37</t>
+          <t>2026/10/12 23:01:15</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -5767,7 +5767,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>125:47:24</t>
+          <t>127:47:02</t>
         </is>
       </c>
       <c r="L92" t="n">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2026/10/12 20:58:30</t>
+          <t>2026/10/12 22:58:30</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -7301,7 +7301,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>82:00:00</t>
+          <t>84:00:00</t>
         </is>
       </c>
       <c r="L118" t="n">
@@ -7876,7 +7876,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>2026/10/12 21:00:34</t>
+          <t>2026/10/12 23:00:34</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>56:58:04</t>
+          <t>58:58:04</t>
         </is>
       </c>
       <c r="L128" t="n">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/10/12 21:22:29</t>
+          <t>2026/10/12 23:22:28</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>10:27:49</t>
+          <t>12:27:48</t>
         </is>
       </c>
       <c r="L130" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/10/12 20:10:55</t>
+          <t>2026/10/12 22:10:55</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>08:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/10/12 20:30:06</t>
+          <t>2026/10/12 22:30:06</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>06:00:00</t>
+          <t>08:00:00</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -8171,31 +8171,90 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026/10/12 21:42:50</t>
+          <t>2026/10/12 23:52:59</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>-33.0873483, -71.362345</t>
+          <t>-33.0872583, -71.3622466</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>-33.08735, -71.36235</t>
+          <t>-33.08726, -71.36225</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>06:00:00</t>
+          <t>08:10:09</t>
         </is>
       </c>
       <c r="L133" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="M133" t="n">
         <v>0</v>
       </c>
       <c r="N133" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>9</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>2026/10/12 20:42:16</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>-33.4362966, -70.6294283</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>-33.43630, -70.62943</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>2026/10/12 22:44:49</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>-33.4362966, -70.6294283</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>-33.43630, -70.62943</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>02:02:33</t>
+        </is>
+      </c>
+      <c r="L134" t="n">
+        <v>0</v>
+      </c>
+      <c r="M134" t="n">
+        <v>0</v>
+      </c>
+      <c r="N134" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8247,10 +8306,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1317.77</v>
+        <v>1341.84</v>
       </c>
       <c r="C2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -8494,13 +8553,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2268.28</v>
+        <v>2268.21</v>
       </c>
       <c r="C15" t="n">
         <v>43</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>145</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-14T09:17Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/10/13 22:54:11</t>
+          <t>2026/10/13 23:54:16</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>166:44:56</t>
+          <t>167:45:01</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/10/13 22:57:28</t>
+          <t>2026/10/13 23:57:28</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>166:00:12</t>
+          <t>167:00:12</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>2026/10/13 22:59:09</t>
+          <t>2026/10/13 23:59:36</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>18:00:00</t>
+          <t>19:00:27</t>
         </is>
       </c>
       <c r="L121" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2026/10/13 22:37:43</t>
+          <t>2026/10/13 23:37:44</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>08:01:52</t>
+          <t>09:01:53</t>
         </is>
       </c>
       <c r="L126" t="n">
@@ -7817,7 +7817,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>2026/10/13 22:40:03</t>
+          <t>2026/10/13 23:39:56</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -7832,7 +7832,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>08:00:04</t>
+          <t>08:59:57</t>
         </is>
       </c>
       <c r="L127" t="n">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/10/13 21:53:08</t>
+          <t>2026/10/13 23:53:08</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L130" t="n">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>2026/10/13 21:36:31</t>
+          <t>2026/10/13 23:36:31</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>00:16:07</t>
+          <t>02:16:07</t>
         </is>
       </c>
       <c r="L142" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-15T08:51Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/10/14 22:54:11</t>
+          <t>2026/10/14 23:54:15</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>166:44:50</t>
+          <t>167:44:54</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026/10/14 22:35:53</t>
+          <t>2026/10/14 23:34:52</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>164:01:28</t>
+          <t>165:00:27</t>
         </is>
       </c>
       <c r="L23" t="n">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>2026/10/14 22:59:09</t>
+          <t>2026/10/14 23:59:09</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>42:00:00</t>
+          <t>43:00:00</t>
         </is>
       </c>
       <c r="L106" t="n">
@@ -6932,7 +6932,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>2026/10/14 22:57:09</t>
+          <t>2026/10/14 23:57:31</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -6947,7 +6947,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>32:21:18</t>
+          <t>33:21:40</t>
         </is>
       </c>
       <c r="L112" t="n">
@@ -6991,7 +6991,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>2026/10/14 22:46:22</t>
+          <t>2026/10/14 23:46:21</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7006,7 +7006,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>32:06:23</t>
+          <t>33:06:22</t>
         </is>
       </c>
       <c r="L113" t="n">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026/10/14 22:20:55</t>
+          <t>2026/10/14 23:20:55</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>08:01:30</t>
+          <t>09:01:30</t>
         </is>
       </c>
       <c r="L134" t="n">
@@ -8289,7 +8289,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>2026/10/14 21:39:13</t>
+          <t>2026/10/14 23:39:13</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -8304,7 +8304,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L135" t="n">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/10/14 22:41:27</t>
+          <t>2026/10/14 23:41:28</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>03:01:00</t>
+          <t>04:01:01</t>
         </is>
       </c>
       <c r="L140" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-16T08:45Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/10/15 22:54:38</t>
+          <t>2026/10/15 23:54:15</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>166:41:23</t>
+          <t>167:41:00</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/10/15 22:35:56</t>
+          <t>2026/10/15 23:35:18</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>166:01:35</t>
+          <t>167:00:57</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>2026/10/15 22:59:17</t>
+          <t>2026/10/15 23:59:36</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>66:00:08</t>
+          <t>67:00:27</t>
         </is>
       </c>
       <c r="L105" t="n">
@@ -6873,7 +6873,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>2026/10/15 22:57:19</t>
+          <t>2026/10/15 23:57:33</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -6888,7 +6888,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>56:21:28</t>
+          <t>57:21:42</t>
         </is>
       </c>
       <c r="L111" t="n">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>2026/10/15 21:32:31</t>
+          <t>2026/10/15 23:32:31</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>03:59:40</t>
+          <t>05:59:40</t>
         </is>
       </c>
       <c r="L138" t="n">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>2026/10/15 21:26:48</t>
+          <t>2026/10/15 23:26:48</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>02:00:17</t>
+          <t>04:00:17</t>
         </is>
       </c>
       <c r="L141" t="n">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>2026/10/15 21:32:23</t>
+          <t>2026/10/15 23:32:23</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L142" t="n">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>2026/10/15 21:38:51</t>
+          <t>2026/10/15 23:38:51</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -8835,7 +8835,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>02:00:22</t>
+          <t>04:00:22</t>
         </is>
       </c>
       <c r="L144" t="n">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>2026/10/15 22:49:25</t>
+          <t>2026/10/15 23:49:25</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>04:01:03</t>
         </is>
       </c>
       <c r="L145" t="n">
@@ -8938,7 +8938,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>2026/10/15 22:19:42</t>
+          <t>2026/10/15 23:19:42</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>02:01:00</t>
+          <t>03:01:00</t>
         </is>
       </c>
       <c r="L146" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-17T08:15Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N142"/>
+  <dimension ref="A1:N141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/10/16 22:13:45</t>
+          <t>2026/10/16 23:13:51</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>166:00:07</t>
+          <t>167:00:13</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/10/16 22:34:31</t>
+          <t>2026/10/16 23:34:53</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>165:57:49</t>
+          <t>166:58:11</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026/10/16 22:32:15</t>
+          <t>2026/10/16 23:32:15</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>06:57:27</t>
+          <t>07:57:27</t>
         </is>
       </c>
       <c r="L134" t="n">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/10/16 21:18:35</t>
+          <t>2026/10/16 23:18:35</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>02:00:08</t>
+          <t>04:00:08</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>2026/10/16 21:47:19</t>
+          <t>2026/10/16 23:47:19</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>02:00:10</t>
+          <t>04:00:10</t>
         </is>
       </c>
       <c r="L141" t="n">
@@ -8668,65 +8668,6 @@
         <v>0</v>
       </c>
       <c r="N141" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>VOLKSWAGEN AMAROK KPDV-13</t>
-        </is>
-      </c>
-      <c r="C142" t="n">
-        <v>8</v>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>Paradas</t>
-        </is>
-      </c>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>2026/10/16 20:53:25</t>
-        </is>
-      </c>
-      <c r="F142" t="inlineStr">
-        <is>
-          <t>-33.484931, -70.772438</t>
-        </is>
-      </c>
-      <c r="G142" t="inlineStr">
-        <is>
-          <t>-33.48493, -70.77244</t>
-        </is>
-      </c>
-      <c r="H142" t="inlineStr">
-        <is>
-          <t>2026/10/16 22:54:52</t>
-        </is>
-      </c>
-      <c r="I142" t="inlineStr">
-        <is>
-          <t>-33.484931, -70.772438</t>
-        </is>
-      </c>
-      <c r="J142" t="inlineStr">
-        <is>
-          <t>-33.48493, -70.77244</t>
-        </is>
-      </c>
-      <c r="K142" t="inlineStr">
-        <is>
-          <t>02:01:27</t>
-        </is>
-      </c>
-      <c r="L142" t="n">
-        <v>0</v>
-      </c>
-      <c r="M142" t="n">
-        <v>0</v>
-      </c>
-      <c r="N142" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9120,13 +9061,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1139.71</v>
+        <v>1141.72</v>
       </c>
       <c r="C20" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>138</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-18T08:33Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N134"/>
+  <dimension ref="A1:N135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/10/17 22:35:49</t>
+          <t>2026/10/17 23:35:17</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>165:59:16</t>
+          <t>166:58:44</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/10/17 22:13:51</t>
+          <t>2026/10/17 23:14:07</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>165:17:14</t>
+          <t>166:17:30</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -5724,7 +5724,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>OPEL COMBO</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -5742,48 +5742,48 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>-33.093635, -71.3554899</t>
+          <t>-33.4098033, -70.6798216</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>-33.09363, -71.35549</t>
+          <t>-33.40980, -70.67982</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>2026/10/13 18:47:33</t>
+          <t>2026/10/13 18:05:55</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>-33.0873383, -71.3622783</t>
+          <t>-33.4122666, -70.6794883</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>-33.08734, -71.36228</t>
+          <t>-33.41227, -70.67949</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>00:55:23</t>
+          <t>00:13:45</t>
         </is>
       </c>
       <c r="L92" t="n">
-        <v>1.34</v>
+        <v>0.28</v>
       </c>
       <c r="M92" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="N92" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -5801,42 +5801,42 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>-33.4098033, -70.6798216</t>
+          <t>-33.093635, -71.3554899</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>-33.40980, -70.67982</t>
+          <t>-33.09363, -71.35549</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>2026/10/13 18:05:55</t>
+          <t>2026/10/13 18:47:33</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>-33.4122666, -70.6794883</t>
+          <t>-33.0873383, -71.3622783</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>-33.41227, -70.67949</t>
+          <t>-33.08734, -71.36228</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>00:13:45</t>
+          <t>00:55:23</t>
         </is>
       </c>
       <c r="L93" t="n">
-        <v>0.28</v>
+        <v>1.34</v>
       </c>
       <c r="M93" t="n">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="N93" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="94">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/10/17 22:27:29</t>
+          <t>2026/10/17 23:27:29</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>11:01:00</t>
+          <t>12:01:00</t>
         </is>
       </c>
       <c r="L130" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/10/17 21:17:48</t>
+          <t>2026/10/17 23:17:48</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>09:22:24</t>
+          <t>11:22:24</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -8255,6 +8255,65 @@
         <v>0</v>
       </c>
       <c r="N134" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TGPS-77</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>7</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>2026/10/17 21:30:59</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>-32.7975866, -70.8870516</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>-32.79759, -70.88705</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>2026/10/17 23:31:01</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>-32.7975866, -70.8870516</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>-32.79759, -70.88705</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>02:00:02</t>
+        </is>
+      </c>
+      <c r="L135" t="n">
+        <v>0</v>
+      </c>
+      <c r="M135" t="n">
+        <v>0</v>
+      </c>
+      <c r="N135" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8306,13 +8365,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1739.03</v>
+        <v>1739</v>
       </c>
       <c r="C2" t="n">
         <v>41</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>142</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-18T22:13Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -5724,7 +5724,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -5742,48 +5742,48 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>-33.4098033, -70.6798216</t>
+          <t>-33.093635, -71.3554899</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>-33.40980, -70.67982</t>
+          <t>-33.09363, -71.35549</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>2026/10/13 18:05:55</t>
+          <t>2026/10/13 18:47:33</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>-33.4122666, -70.6794883</t>
+          <t>-33.0873383, -71.3622783</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>-33.41227, -70.67949</t>
+          <t>-33.08734, -71.36228</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>00:13:45</t>
+          <t>00:55:23</t>
         </is>
       </c>
       <c r="L92" t="n">
-        <v>0.28</v>
+        <v>1.34</v>
       </c>
       <c r="M92" t="n">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="N92" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>OPEL COMBO</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -5801,42 +5801,42 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>-33.093635, -71.3554899</t>
+          <t>-33.4098033, -70.6798216</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>-33.09363, -71.35549</t>
+          <t>-33.40980, -70.67982</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>2026/10/13 18:47:33</t>
+          <t>2026/10/13 18:05:55</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>-33.0873383, -71.3622783</t>
+          <t>-33.4122666, -70.6794883</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>-33.08734, -71.36228</t>
+          <t>-33.41227, -70.67949</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>00:55:23</t>
+          <t>00:13:45</t>
         </is>
       </c>
       <c r="L93" t="n">
-        <v>1.34</v>
+        <v>0.28</v>
       </c>
       <c r="M93" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="N93" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-19T09:35Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N136"/>
+  <dimension ref="A1:N137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/10/18 22:35:35</t>
+          <t>2026/10/18 23:34:28</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>166:00:31</t>
+          <t>166:59:24</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/10/18 21:36:45</t>
+          <t>2026/10/18 23:36:45</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>08:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -8373,6 +8373,65 @@
         <v>0</v>
       </c>
       <c r="N136" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>7</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>2026/10/18 21:41:59</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>-33.4762049, -70.6984233</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>-33.47620, -70.69842</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>2026/10/18 23:42:22</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>-33.4762049, -70.6984233</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>-33.47620, -70.69842</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>02:00:23</t>
+        </is>
+      </c>
+      <c r="L137" t="n">
+        <v>0</v>
+      </c>
+      <c r="M137" t="n">
+        <v>0</v>
+      </c>
+      <c r="N137" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8652,13 +8711,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1107.17</v>
+        <v>1107.15</v>
       </c>
       <c r="C14" t="n">
         <v>69</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>128</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-20T09:07Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -7994,7 +7994,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/10/19 22:31:25</t>
+          <t>2026/10/19 23:31:59</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>91:42:22</t>
+          <t>92:42:56</t>
         </is>
       </c>
       <c r="L130" t="n">
@@ -8997,7 +8997,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>2026/10/19 22:36:25</t>
+          <t>2026/10/19 23:36:25</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>05:01:20</t>
+          <t>06:01:20</t>
         </is>
       </c>
       <c r="L147" t="n">
@@ -9233,7 +9233,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>2026/10/19 21:41:27</t>
+          <t>2026/10/19 23:41:27</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L151" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-21T09:07Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -8348,7 +8348,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026/10/20 22:55:02</t>
+          <t>2026/10/20 23:54:54</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>11:59:45</t>
+          <t>12:59:37</t>
         </is>
       </c>
       <c r="L136" t="n">
@@ -8525,7 +8525,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>2026/10/20 21:56:27</t>
+          <t>2026/10/20 23:56:27</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -8540,7 +8540,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>06:00:00</t>
+          <t>08:00:00</t>
         </is>
       </c>
       <c r="L139" t="n">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026/10/20 22:24:05</t>
+          <t>2026/10/20 23:24:05</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -8776,7 +8776,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>03:01:04</t>
+          <t>04:01:04</t>
         </is>
       </c>
       <c r="L143" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-22T09:09Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -8407,7 +8407,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2026/10/21 22:41:17</t>
+          <t>2026/10/21 23:41:16</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>11:01:58</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="L137" t="n">
@@ -8525,7 +8525,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>2026/10/21 21:51:14</t>
+          <t>2026/10/21 23:51:14</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -8540,7 +8540,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>02:00:07</t>
+          <t>04:00:07</t>
         </is>
       </c>
       <c r="L139" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-23T09:06Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1799,7 +1799,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026/10/22 22:31:23</t>
+          <t>2026/10/22 23:31:38</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>163:42:20</t>
+          <t>164:42:35</t>
         </is>
       </c>
       <c r="L25" t="n">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026/10/22 22:34:30</t>
+          <t>2026/10/22 23:35:07</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>34:55:11</t>
+          <t>35:55:48</t>
         </is>
       </c>
       <c r="L136" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026/10/22 21:47:08</t>
+          <t>2026/10/22 23:47:08</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>04:00:23</t>
+          <t>06:00:23</t>
         </is>
       </c>
       <c r="L159" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/10/22 22:44:20</t>
+          <t>2026/10/22 23:44:20</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>04:49:45</t>
+          <t>05:49:45</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>2026/10/22 21:44:31</t>
+          <t>2026/10/22 23:44:31</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>02:04:53</t>
+          <t>04:04:53</t>
         </is>
       </c>
       <c r="L164" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-24T08:39Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/10/23 22:40:16</t>
+          <t>2026/10/23 23:40:16</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>166:26:08</t>
+          <t>167:26:08</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/10/23 22:31:24</t>
+          <t>2026/10/23 23:31:38</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>165:41:53</t>
+          <t>166:42:07</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -6991,7 +6991,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>2026/10/23 22:57:38</t>
+          <t>2026/10/23 23:57:15</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7006,7 +7006,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>69:00:00</t>
+          <t>69:59:37</t>
         </is>
       </c>
       <c r="L113" t="n">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>2026/10/23 21:23:25</t>
+          <t>2026/10/23 23:23:25</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>01:53:52</t>
+          <t>03:53:52</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>2026/10/23 22:42:50</t>
+          <t>2026/10/23 23:42:50</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -9897,7 +9897,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>00:21:32</t>
+          <t>01:21:32</t>
         </is>
       </c>
       <c r="L162" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-25T08:57Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/10/24 22:40:20</t>
+          <t>2026/10/24 23:39:57</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>166:26:29</t>
+          <t>167:26:06</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/10/24 22:31:21</t>
+          <t>2026/10/24 23:31:22</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>165:42:18</t>
+          <t>166:42:19</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -6873,7 +6873,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>2026/10/24 22:57:37</t>
+          <t>2026/10/24 23:57:14</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -6888,7 +6888,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>92:59:59</t>
+          <t>93:59:36</t>
         </is>
       </c>
       <c r="L111" t="n">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2026/10/24 22:34:36</t>
+          <t>2026/10/24 23:34:26</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>34:19:17</t>
+          <t>35:19:07</t>
         </is>
       </c>
       <c r="L154" t="n">
@@ -9528,7 +9528,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>2026/10/24 21:20:38</t>
+          <t>2026/10/24 23:20:38</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>30:03:03</t>
+          <t>32:03:03</t>
         </is>
       </c>
       <c r="L156" t="n">
@@ -9587,7 +9587,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>2026/10/24 21:40:11</t>
+          <t>2026/10/24 23:40:11</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -9602,7 +9602,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="L157" t="n">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>2026/10/24 21:20:52</t>
+          <t>2026/10/24 23:20:52</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>04:00:11</t>
+          <t>06:00:11</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026/10/24 21:23:43</t>
+          <t>2026/10/24 23:23:43</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>02:17:38</t>
+          <t>04:17:38</t>
         </is>
       </c>
       <c r="L159" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-26T09:42Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N163"/>
+  <dimension ref="A1:N164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/10/25 22:40:20</t>
+          <t>2026/10/25 23:39:57</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>166:26:42</t>
+          <t>167:26:19</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/10/25 22:31:47</t>
+          <t>2026/10/25 23:31:21</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>165:42:44</t>
+          <t>166:42:18</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>2026/10/25 22:57:37</t>
+          <t>2026/10/25 23:57:14</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>116:59:59</t>
+          <t>117:59:36</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -9528,7 +9528,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>2026/10/25 22:34:51</t>
+          <t>2026/10/25 23:34:35</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>58:19:32</t>
+          <t>59:19:16</t>
         </is>
       </c>
       <c r="L156" t="n">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>2026/10/25 21:50:22</t>
+          <t>2026/10/25 23:50:22</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>54:32:47</t>
+          <t>56:32:47</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026/10/25 21:20:52</t>
+          <t>2026/10/25 23:20:52</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>28:00:11</t>
+          <t>30:00:11</t>
         </is>
       </c>
       <c r="L159" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/10/25 21:59:09</t>
+          <t>2026/10/25 23:59:09</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -9966,6 +9966,65 @@
         <v>0</v>
       </c>
       <c r="N163" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>4</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>2026/10/25 22:26:53</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>-32.841619, -70.93683</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>-32.84162, -70.93683</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>2026/10/25 23:27:54</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>-32.841619, -70.93683</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>-32.84162, -70.93683</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>01:01:01</t>
+        </is>
+      </c>
+      <c r="L164" t="n">
+        <v>0</v>
+      </c>
+      <c r="M164" t="n">
+        <v>0</v>
+      </c>
+      <c r="N164" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10359,13 +10418,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1175.15</v>
+        <v>1175.14</v>
       </c>
       <c r="C20" t="n">
         <v>57</v>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
         <v>135</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-10-27T09:36Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -4690,7 +4690,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>2026/10/26 22:57:38</t>
+          <t>2026/10/26 23:57:21</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>141:00:00</t>
+          <t>141:59:43</t>
         </is>
       </c>
       <c r="L74" t="n">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>2026/10/26 21:57:12</t>
+          <t>2026/10/26 23:57:12</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -9838,7 +9838,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>02:00:13</t>
+          <t>04:00:13</t>
         </is>
       </c>
       <c r="L161" t="n">

</xml_diff>